<commit_message>
Add Suffolk County towns + bulk Excel parsers for free cash and debt
- Add Boston, Revere, Winthrop — dataset now covers 50 towns (all of
  Suffolk County: Chelsea already present)
- Parse CFC_PerBudg.xlsx: free_cash_pct_of_budget for all 351 MA
  municipalities (best available year)
- Parse municipaldebt2022.xlsx: debt_per_capita = total outstanding
  debt / Census population for 336 municipalities
- Extend HTML patcher to sync inc10yr, pop10yr, med_inc, free_cash,
  debt_pc, bond on every update_all.py run
- New scores: Boston 77, Revere 65, Winthrop 68

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/civica_value_scores.xlsx
+++ b/civica_value_scores.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -690,10 +690,10 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>91.40000000000001</v>
+        <v>92.8</v>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
@@ -712,14 +712,14 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>Haverhill</t>
+          <t>Revere</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>85</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
@@ -727,37 +727,37 @@
         </is>
       </c>
       <c r="E3" s="10" t="n">
-        <v>497568</v>
+        <v>440000</v>
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Suffolk</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Uxbridge</t>
+          <t>Haverhill</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>65</v>
-      </c>
-      <c r="C4" s="12" t="n">
-        <v>81.8</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>Good Value</t>
+        <v>71</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Great Value</t>
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>487277</v>
+        <v>497568</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Worcester</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
@@ -768,10 +768,10 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>79.7</v>
+        <v>80.8</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -790,14 +790,14 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Lynn</t>
+          <t>Winthrop</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
         <v>68</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>77.5</v>
+        <v>80.2</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
@@ -805,25 +805,25 @@
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>537825</v>
+        <v>520000</v>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Suffolk</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Amesbury</t>
+          <t>Lynn</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
         <v>70</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>75.3</v>
+        <v>79.8</v>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="E7" s="10" t="n">
-        <v>570013</v>
+        <v>537825</v>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
@@ -842,14 +842,14 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Uxbridge</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>74</v>
+        <v>79.3</v>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
@@ -857,25 +857,25 @@
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>505101</v>
+        <v>487277</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Suffolk</t>
+          <t>Worcester</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Merrimac</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>69.8</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
@@ -883,11 +883,11 @@
         </is>
       </c>
       <c r="E9" s="10" t="n">
-        <v>597359</v>
+        <v>505101</v>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Suffolk</t>
         </is>
       </c>
     </row>
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>69.59999999999999</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
@@ -920,14 +920,14 @@
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Salisbury</t>
+          <t>Amesbury</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>67.59999999999999</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
         </is>
       </c>
       <c r="E11" s="10" t="n">
-        <v>589785</v>
+        <v>570013</v>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
@@ -946,14 +946,14 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Woburn</t>
+          <t>Merrimac</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C12" s="12" t="n">
-        <v>67</v>
+        <v>70.8</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
@@ -961,25 +961,25 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>704405</v>
+        <v>597359</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Saugus</t>
+          <t>Woburn</t>
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>66.90000000000001</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
@@ -987,25 +987,25 @@
         </is>
       </c>
       <c r="E13" s="10" t="n">
-        <v>650624</v>
+        <v>704405</v>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Danvers</t>
+          <t>Saugus</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>66.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>674241</v>
+        <v>650624</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -1024,14 +1024,14 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Beverly</t>
+          <t>Salisbury</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>65.2</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="E15" s="10" t="n">
-        <v>696077</v>
+        <v>589785</v>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
@@ -1050,26 +1050,26 @@
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Burlington</t>
+          <t>Danvers</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>85</v>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>63.2</v>
-      </c>
-      <c r="D16" s="15" t="inlineStr">
-        <is>
-          <t>Fair Market</t>
+        <v>73</v>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>824833</v>
+        <v>674241</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
@@ -1080,14 +1080,14 @@
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>66</v>
-      </c>
-      <c r="C17" s="14" t="n">
-        <v>62.4</v>
-      </c>
-      <c r="D17" s="15" t="inlineStr">
-        <is>
-          <t>Fair Market</t>
+        <v>70</v>
+      </c>
+      <c r="C17" s="12" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E17" s="10" t="n">
@@ -1102,40 +1102,40 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Wakefield</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
         <v>77</v>
       </c>
-      <c r="C18" s="14" t="n">
-        <v>62.4</v>
-      </c>
-      <c r="D18" s="15" t="inlineStr">
-        <is>
-          <t>Fair Market</t>
+      <c r="C18" s="12" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>756484</v>
+        <v>720000</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Suffolk</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>North Andover</t>
+          <t>Beverly</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C19" s="14" t="n">
-        <v>59.6</v>
+        <v>64.3</v>
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="E19" s="10" t="n">
-        <v>760639</v>
+        <v>696077</v>
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
@@ -1154,14 +1154,14 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Gloucester</t>
+          <t>Burlington</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="C20" s="14" t="n">
-        <v>57.5</v>
+        <v>63.2</v>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>693415</v>
+        <v>824833</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Peabody</t>
+          <t>Wakefield</t>
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="C21" s="14" t="n">
-        <v>57.3</v>
+        <v>63.2</v>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
@@ -1195,25 +1195,25 @@
         </is>
       </c>
       <c r="E21" s="10" t="n">
-        <v>652390</v>
+        <v>756484</v>
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Georgetown</t>
+          <t>North Andover</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="C22" s="14" t="n">
-        <v>57.1</v>
+        <v>60.4</v>
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>708796</v>
+        <v>760639</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
@@ -1236,10 +1236,10 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C23" s="14" t="n">
-        <v>57</v>
+        <v>58.6</v>
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
@@ -1258,14 +1258,14 @@
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Rowley</t>
+          <t>Peabody</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C24" s="14" t="n">
-        <v>56.8</v>
+        <v>58.3</v>
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>733628</v>
+        <v>652390</v>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
@@ -1284,14 +1284,14 @@
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>Georgetown</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="C25" s="14" t="n">
-        <v>56.7</v>
+        <v>57.9</v>
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="E25" s="10" t="n">
-        <v>844034</v>
+        <v>708796</v>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Andover</t>
+          <t>Ipswich</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="C26" s="14" t="n">
-        <v>55.8</v>
+        <v>57.4</v>
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
@@ -1325,7 +1325,7 @@
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>911128</v>
+        <v>790546</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
@@ -1336,14 +1336,14 @@
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Ipswich</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C27" s="14" t="n">
-        <v>55.8</v>
+        <v>57.4</v>
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
@@ -1351,25 +1351,25 @@
         </is>
       </c>
       <c r="E27" s="10" t="n">
-        <v>790546</v>
+        <v>844034</v>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Swampscott</t>
+          <t>Rowley</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C28" s="14" t="n">
-        <v>53.8</v>
+        <v>56.8</v>
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
@@ -1377,7 +1377,7 @@
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>763080</v>
+        <v>733628</v>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
@@ -1388,14 +1388,14 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Newburyport</t>
+          <t>Gloucester</t>
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C29" s="14" t="n">
-        <v>52.9</v>
+        <v>56.6</v>
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="E29" s="10" t="n">
-        <v>845604</v>
+        <v>693415</v>
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
@@ -1414,14 +1414,14 @@
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Middleton</t>
+          <t>Andover</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C30" s="14" t="n">
-        <v>52.4</v>
+        <v>55.8</v>
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>819582</v>
+        <v>911128</v>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
@@ -1440,14 +1440,14 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Somerville</t>
+          <t>Swampscott</t>
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C31" s="14" t="n">
-        <v>52.2</v>
+        <v>55.4</v>
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
@@ -1455,25 +1455,25 @@
         </is>
       </c>
       <c r="E31" s="10" t="n">
-        <v>892143</v>
+        <v>763080</v>
       </c>
       <c r="F31" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Hamilton</t>
+          <t>Middleton</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C32" s="14" t="n">
-        <v>51.1</v>
+        <v>55.4</v>
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>827397</v>
+        <v>819582</v>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
@@ -1492,14 +1492,14 @@
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Rockport</t>
+          <t>Hamilton</t>
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C33" s="14" t="n">
-        <v>50</v>
+        <v>53.3</v>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="E33" s="10" t="n">
-        <v>834071</v>
+        <v>827397</v>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
@@ -1518,22 +1518,22 @@
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Marblehead</t>
+          <t>Newbury</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>78</v>
-      </c>
-      <c r="C34" s="16" t="n">
-        <v>49.8</v>
-      </c>
-      <c r="D34" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>72</v>
+      </c>
+      <c r="C34" s="14" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>959425</v>
+        <v>844611</v>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
@@ -1544,22 +1544,22 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Rockport</t>
         </is>
       </c>
       <c r="B35" s="9" t="n">
-        <v>67</v>
-      </c>
-      <c r="C35" s="16" t="n">
-        <v>49.7</v>
-      </c>
-      <c r="D35" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>71</v>
+      </c>
+      <c r="C35" s="14" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E35" s="10" t="n">
-        <v>827029</v>
+        <v>834071</v>
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
@@ -1570,22 +1570,22 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Newbury</t>
+          <t>Newburyport</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>68</v>
-      </c>
-      <c r="C36" s="16" t="n">
-        <v>49.4</v>
-      </c>
-      <c r="D36" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>71</v>
+      </c>
+      <c r="C36" s="14" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>844611</v>
+        <v>845604</v>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
@@ -1596,22 +1596,22 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>Cambridge</t>
+          <t>Somerville</t>
         </is>
       </c>
       <c r="B37" s="9" t="n">
-        <v>79</v>
-      </c>
-      <c r="C37" s="16" t="n">
-        <v>48.7</v>
-      </c>
-      <c r="D37" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>75</v>
+      </c>
+      <c r="C37" s="14" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E37" s="10" t="n">
-        <v>995293</v>
+        <v>892143</v>
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
@@ -1622,22 +1622,22 @@
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>West Newbury</t>
+          <t>Marblehead</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>67</v>
-      </c>
-      <c r="C38" s="16" t="n">
-        <v>47.7</v>
-      </c>
-      <c r="D38" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>79</v>
+      </c>
+      <c r="C38" s="14" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>861236</v>
+        <v>959425</v>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
@@ -1648,48 +1648,48 @@
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>Arlington</t>
+          <t>West Newbury</t>
         </is>
       </c>
       <c r="B39" s="9" t="n">
-        <v>76</v>
-      </c>
-      <c r="C39" s="16" t="n">
-        <v>46.3</v>
-      </c>
-      <c r="D39" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>71</v>
+      </c>
+      <c r="C39" s="14" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E39" s="10" t="n">
-        <v>1005584</v>
+        <v>861236</v>
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Topsfield</t>
+          <t>Essex</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>66</v>
-      </c>
-      <c r="C40" s="16" t="n">
-        <v>45</v>
-      </c>
-      <c r="D40" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>68</v>
+      </c>
+      <c r="C40" s="14" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>898745</v>
+        <v>827029</v>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
@@ -1700,14 +1700,14 @@
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>Lynnfield</t>
+          <t>Cambridge</t>
         </is>
       </c>
       <c r="B41" s="9" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C41" s="16" t="n">
-        <v>44</v>
+        <v>48.7</v>
       </c>
       <c r="D41" s="17" t="inlineStr">
         <is>
@@ -1715,25 +1715,25 @@
         </is>
       </c>
       <c r="E41" s="10" t="n">
-        <v>1018229</v>
+        <v>995293</v>
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Wenham</t>
+          <t>Boxford</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C42" s="16" t="n">
-        <v>43.8</v>
+        <v>45.9</v>
       </c>
       <c r="D42" s="17" t="inlineStr">
         <is>
@@ -1741,7 +1741,7 @@
         </is>
       </c>
       <c r="E42" s="6" t="n">
-        <v>938834</v>
+        <v>989433</v>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
@@ -1752,14 +1752,14 @@
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>Boxford</t>
+          <t>Topsfield</t>
         </is>
       </c>
       <c r="B43" s="9" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C43" s="16" t="n">
-        <v>43.4</v>
+        <v>45.7</v>
       </c>
       <c r="D43" s="17" t="inlineStr">
         <is>
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="E43" s="10" t="n">
-        <v>989433</v>
+        <v>898745</v>
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
@@ -1778,14 +1778,14 @@
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Nahant</t>
+          <t>Wenham</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="C44" s="16" t="n">
-        <v>39.4</v>
+        <v>45.7</v>
       </c>
       <c r="D44" s="17" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="E44" s="6" t="n">
-        <v>903532</v>
+        <v>938834</v>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
@@ -1804,14 +1804,14 @@
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Manchester-by-the-Sea</t>
+          <t>Lynnfield</t>
         </is>
       </c>
       <c r="B45" s="9" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C45" s="16" t="n">
-        <v>36.2</v>
+        <v>45.2</v>
       </c>
       <c r="D45" s="17" t="inlineStr">
         <is>
@@ -1819,7 +1819,7 @@
         </is>
       </c>
       <c r="E45" s="10" t="n">
-        <v>1183983</v>
+        <v>1018229</v>
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
@@ -1830,22 +1830,22 @@
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Belmont</t>
+          <t>Arlington</t>
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>76</v>
-      </c>
-      <c r="C46" s="18" t="n">
-        <v>33.8</v>
-      </c>
-      <c r="D46" s="19" t="inlineStr">
-        <is>
-          <t>Luxury</t>
+        <v>74</v>
+      </c>
+      <c r="C46" s="16" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="D46" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>1377983</v>
+        <v>1005584</v>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
@@ -1856,50 +1856,128 @@
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>Winchester</t>
+          <t>Nahant</t>
         </is>
       </c>
       <c r="B47" s="9" t="n">
-        <v>79</v>
-      </c>
-      <c r="C47" s="18" t="n">
-        <v>33.4</v>
-      </c>
-      <c r="D47" s="19" t="inlineStr">
-        <is>
-          <t>Luxury</t>
+        <v>59</v>
+      </c>
+      <c r="C47" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
         </is>
       </c>
       <c r="E47" s="10" t="n">
-        <v>1449988</v>
+        <v>903532</v>
       </c>
       <c r="F47" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>Manchester-by-the-Sea</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C48" s="16" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>1183983</v>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>Belmont</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="C49" s="18" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="D49" s="19" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="n">
+        <v>1377983</v>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
           <t>Lexington</t>
         </is>
       </c>
-      <c r="B48" s="3" t="n">
-        <v>78</v>
-      </c>
-      <c r="C48" s="18" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="D48" s="19" t="inlineStr">
+      <c r="B50" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="C50" s="18" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="D50" s="19" t="inlineStr">
         <is>
           <t>Luxury</t>
         </is>
       </c>
-      <c r="E48" s="6" t="n">
+      <c r="E50" s="6" t="n">
         <v>1469802</v>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Winchester</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="n">
+        <v>76</v>
+      </c>
+      <c r="C51" s="18" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="D51" s="19" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="n">
+        <v>1449988</v>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
         <is>
           <t>Middlesex</t>
         </is>

</xml_diff>

<commit_message>
Add 10 Middlesex towns, bring total to 60 cities/towns
Newton (83), Natick (80), Concord (80), Watertown (79), Acton (79),
Stoneham (79), Waltham (74), Malden (74), Framingham (69), Everett (67).

- Updated site badge, map subtitle, and stats counter from 47 → 60
- Added ZHVI and DISTRICT_MAP entries for all 10 new towns
- Regenerated civica_value_scores.xlsx with all 60 towns

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/civica_value_scores.xlsx
+++ b/civica_value_scores.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -764,40 +764,40 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Methuen</t>
+          <t>Malden</t>
         </is>
       </c>
       <c r="B5" s="9" t="n">
         <v>74</v>
       </c>
-      <c r="C5" s="12" t="n">
-        <v>80.8</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>Good Value</t>
+      <c r="C5" s="4" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Great Value</t>
         </is>
       </c>
       <c r="E5" s="10" t="n">
-        <v>561211</v>
+        <v>545000</v>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Winthrop</t>
+          <t>Methuen</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>80.2</v>
+        <v>80.8</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
@@ -805,25 +805,25 @@
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>520000</v>
+        <v>561211</v>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Suffolk</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Lynn</t>
+          <t>Winthrop</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>79.8</v>
+        <v>80.2</v>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
@@ -831,25 +831,25 @@
         </is>
       </c>
       <c r="E7" s="10" t="n">
-        <v>537825</v>
+        <v>520000</v>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Suffolk</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Uxbridge</t>
+          <t>Lynn</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>79.3</v>
+        <v>79.8</v>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
@@ -857,25 +857,25 @@
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>487277</v>
+        <v>537825</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Worcester</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Uxbridge</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>78.90000000000001</v>
+        <v>79.3</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
@@ -883,25 +883,25 @@
         </is>
       </c>
       <c r="E9" s="10" t="n">
-        <v>505101</v>
+        <v>487277</v>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Suffolk</t>
+          <t>Worcester</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Salem</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>73.90000000000001</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>572734</v>
+        <v>505101</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Suffolk</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Amesbury</t>
+          <t>Everett</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>73.09999999999999</v>
+        <v>77.5</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
@@ -935,25 +935,25 @@
         </is>
       </c>
       <c r="E11" s="10" t="n">
-        <v>570013</v>
+        <v>530000</v>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Merrimac</t>
+          <t>Salem</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
         <v>69</v>
       </c>
       <c r="C12" s="12" t="n">
-        <v>70.8</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>597359</v>
+        <v>572734</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
@@ -972,14 +972,14 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Woburn</t>
+          <t>Framingham</t>
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>67.90000000000001</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="E13" s="10" t="n">
-        <v>704405</v>
+        <v>575000</v>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
@@ -998,14 +998,14 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Saugus</t>
+          <t>Amesbury</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>67.8</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>650624</v>
+        <v>570013</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -1024,14 +1024,14 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Salisbury</t>
+          <t>Merrimac</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>67.59999999999999</v>
+        <v>70.8</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="E15" s="10" t="n">
-        <v>589785</v>
+        <v>597359</v>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
@@ -1050,14 +1050,14 @@
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Danvers</t>
+          <t>Stoneham</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>66.40000000000001</v>
+        <v>70.2</v>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
@@ -1065,25 +1065,25 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>674241</v>
+        <v>690000</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Groveland</t>
+          <t>Danvers</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>66.2</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="E17" s="10" t="n">
-        <v>648353</v>
+        <v>674241</v>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
@@ -1102,14 +1102,14 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Woburn</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C18" s="12" t="n">
-        <v>65.59999999999999</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
@@ -1117,33 +1117,33 @@
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>720000</v>
+        <v>704405</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Suffolk</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Beverly</t>
+          <t>Saugus</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>73</v>
-      </c>
-      <c r="C19" s="14" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="D19" s="15" t="inlineStr">
-        <is>
-          <t>Fair Market</t>
+        <v>72</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E19" s="10" t="n">
-        <v>696077</v>
+        <v>650624</v>
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
@@ -1154,92 +1154,92 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Burlington</t>
+          <t>Salisbury</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>85</v>
-      </c>
-      <c r="C20" s="14" t="n">
-        <v>63.2</v>
-      </c>
-      <c r="D20" s="15" t="inlineStr">
-        <is>
-          <t>Fair Market</t>
+        <v>65</v>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>824833</v>
+        <v>589785</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Wakefield</t>
+          <t>Groveland</t>
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>78</v>
-      </c>
-      <c r="C21" s="14" t="n">
-        <v>63.2</v>
-      </c>
-      <c r="D21" s="15" t="inlineStr">
-        <is>
-          <t>Fair Market</t>
+        <v>70</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E21" s="10" t="n">
-        <v>756484</v>
+        <v>648353</v>
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>North Andover</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>75</v>
-      </c>
-      <c r="C22" s="14" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>Fair Market</t>
+        <v>77</v>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>760639</v>
+        <v>720000</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Suffolk</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Medford</t>
+          <t>Beverly</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C23" s="14" t="n">
-        <v>58.6</v>
+        <v>64.3</v>
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
@@ -1247,25 +1247,25 @@
         </is>
       </c>
       <c r="E23" s="10" t="n">
-        <v>784462</v>
+        <v>696077</v>
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Peabody</t>
+          <t>Natick</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="C24" s="14" t="n">
-        <v>58.3</v>
+        <v>63.3</v>
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
@@ -1273,25 +1273,25 @@
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>652390</v>
+        <v>775000</v>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Georgetown</t>
+          <t>Burlington</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="C25" s="14" t="n">
-        <v>57.9</v>
+        <v>63.2</v>
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="E25" s="10" t="n">
-        <v>708796</v>
+        <v>824833</v>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Ipswich</t>
+          <t>Wakefield</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C26" s="14" t="n">
-        <v>57.4</v>
+        <v>63.2</v>
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
@@ -1325,25 +1325,25 @@
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>790546</v>
+        <v>756484</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>Waltham</t>
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C27" s="14" t="n">
-        <v>57.4</v>
+        <v>63</v>
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
         </is>
       </c>
       <c r="E27" s="10" t="n">
-        <v>844034</v>
+        <v>720000</v>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
@@ -1362,14 +1362,14 @@
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Rowley</t>
+          <t>North Andover</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C28" s="14" t="n">
-        <v>56.8</v>
+        <v>60.4</v>
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
@@ -1377,7 +1377,7 @@
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>733628</v>
+        <v>760639</v>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
@@ -1388,14 +1388,14 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Gloucester</t>
+          <t>Medford</t>
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="C29" s="14" t="n">
-        <v>56.6</v>
+        <v>58.6</v>
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
@@ -1403,25 +1403,25 @@
         </is>
       </c>
       <c r="E29" s="10" t="n">
-        <v>693415</v>
+        <v>784462</v>
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Andover</t>
+          <t>Peabody</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="C30" s="14" t="n">
-        <v>55.8</v>
+        <v>58.3</v>
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>911128</v>
+        <v>652390</v>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
@@ -1440,14 +1440,14 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Swampscott</t>
+          <t>Georgetown</t>
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C31" s="14" t="n">
-        <v>55.4</v>
+        <v>57.9</v>
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="E31" s="10" t="n">
-        <v>763080</v>
+        <v>708796</v>
       </c>
       <c r="F31" s="11" t="inlineStr">
         <is>
@@ -1466,14 +1466,14 @@
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Middleton</t>
+          <t>Watertown</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C32" s="14" t="n">
-        <v>55.4</v>
+        <v>57.7</v>
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
@@ -1481,25 +1481,25 @@
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>819582</v>
+        <v>840000</v>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Hamilton</t>
+          <t>Acton</t>
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C33" s="14" t="n">
-        <v>53.3</v>
+        <v>57.7</v>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
@@ -1507,25 +1507,25 @@
         </is>
       </c>
       <c r="E33" s="10" t="n">
-        <v>827397</v>
+        <v>840000</v>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Newbury</t>
+          <t>Ipswich</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C34" s="14" t="n">
-        <v>52.3</v>
+        <v>57.4</v>
       </c>
       <c r="D34" s="15" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>844611</v>
+        <v>790546</v>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
@@ -1544,14 +1544,14 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>Rockport</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B35" s="9" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C35" s="14" t="n">
-        <v>52.2</v>
+        <v>57.4</v>
       </c>
       <c r="D35" s="15" t="inlineStr">
         <is>
@@ -1559,25 +1559,25 @@
         </is>
       </c>
       <c r="E35" s="10" t="n">
-        <v>834071</v>
+        <v>844034</v>
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Newburyport</t>
+          <t>Rowley</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C36" s="14" t="n">
-        <v>51.5</v>
+        <v>56.8</v>
       </c>
       <c r="D36" s="15" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>845604</v>
+        <v>733628</v>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
@@ -1596,14 +1596,14 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>Somerville</t>
+          <t>Gloucester</t>
         </is>
       </c>
       <c r="B37" s="9" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C37" s="14" t="n">
-        <v>51.5</v>
+        <v>56.6</v>
       </c>
       <c r="D37" s="15" t="inlineStr">
         <is>
@@ -1611,25 +1611,25 @@
         </is>
       </c>
       <c r="E37" s="10" t="n">
-        <v>892143</v>
+        <v>693415</v>
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Marblehead</t>
+          <t>Andover</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C38" s="14" t="n">
-        <v>50.5</v>
+        <v>55.8</v>
       </c>
       <c r="D38" s="15" t="inlineStr">
         <is>
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>959425</v>
+        <v>911128</v>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
@@ -1648,14 +1648,14 @@
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>West Newbury</t>
+          <t>Swampscott</t>
         </is>
       </c>
       <c r="B39" s="9" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C39" s="14" t="n">
-        <v>50.5</v>
+        <v>55.4</v>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
@@ -1663,7 +1663,7 @@
         </is>
       </c>
       <c r="E39" s="10" t="n">
-        <v>861236</v>
+        <v>763080</v>
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
@@ -1674,14 +1674,14 @@
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middleton</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C40" s="14" t="n">
-        <v>50.4</v>
+        <v>55.4</v>
       </c>
       <c r="D40" s="15" t="inlineStr">
         <is>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>827029</v>
+        <v>819582</v>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
@@ -1700,48 +1700,48 @@
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>Cambridge</t>
+          <t>Hamilton</t>
         </is>
       </c>
       <c r="B41" s="9" t="n">
-        <v>79</v>
-      </c>
-      <c r="C41" s="16" t="n">
-        <v>48.7</v>
-      </c>
-      <c r="D41" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>72</v>
+      </c>
+      <c r="C41" s="14" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E41" s="10" t="n">
-        <v>995293</v>
+        <v>827397</v>
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Boxford</t>
+          <t>Newbury</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>74</v>
-      </c>
-      <c r="C42" s="16" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="D42" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>72</v>
+      </c>
+      <c r="C42" s="14" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E42" s="6" t="n">
-        <v>989433</v>
+        <v>844611</v>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
@@ -1752,22 +1752,22 @@
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>Topsfield</t>
+          <t>Rockport</t>
         </is>
       </c>
       <c r="B43" s="9" t="n">
-        <v>67</v>
-      </c>
-      <c r="C43" s="16" t="n">
-        <v>45.7</v>
-      </c>
-      <c r="D43" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>71</v>
+      </c>
+      <c r="C43" s="14" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E43" s="10" t="n">
-        <v>898745</v>
+        <v>834071</v>
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
@@ -1778,22 +1778,22 @@
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Wenham</t>
+          <t>Newburyport</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>70</v>
-      </c>
-      <c r="C44" s="16" t="n">
-        <v>45.7</v>
-      </c>
-      <c r="D44" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>71</v>
+      </c>
+      <c r="C44" s="14" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E44" s="6" t="n">
-        <v>938834</v>
+        <v>845604</v>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
@@ -1804,74 +1804,74 @@
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Lynnfield</t>
+          <t>Somerville</t>
         </is>
       </c>
       <c r="B45" s="9" t="n">
         <v>75</v>
       </c>
-      <c r="C45" s="16" t="n">
-        <v>45.2</v>
-      </c>
-      <c r="D45" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+      <c r="C45" s="14" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E45" s="10" t="n">
-        <v>1018229</v>
+        <v>892143</v>
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Arlington</t>
+          <t>Marblehead</t>
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>74</v>
-      </c>
-      <c r="C46" s="16" t="n">
-        <v>45.1</v>
-      </c>
-      <c r="D46" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>79</v>
+      </c>
+      <c r="C46" s="14" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>1005584</v>
+        <v>959425</v>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>Nahant</t>
+          <t>West Newbury</t>
         </is>
       </c>
       <c r="B47" s="9" t="n">
-        <v>59</v>
-      </c>
-      <c r="C47" s="16" t="n">
-        <v>40</v>
-      </c>
-      <c r="D47" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>71</v>
+      </c>
+      <c r="C47" s="14" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E47" s="10" t="n">
-        <v>903532</v>
+        <v>861236</v>
       </c>
       <c r="F47" s="11" t="inlineStr">
         <is>
@@ -1882,22 +1882,22 @@
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Manchester-by-the-Sea</t>
+          <t>Essex</t>
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>70</v>
-      </c>
-      <c r="C48" s="16" t="n">
-        <v>36.2</v>
-      </c>
-      <c r="D48" s="17" t="inlineStr">
-        <is>
-          <t>Premium</t>
+        <v>68</v>
+      </c>
+      <c r="C48" s="14" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E48" s="6" t="n">
-        <v>1183983</v>
+        <v>827029</v>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
@@ -1908,22 +1908,22 @@
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>Belmont</t>
+          <t>Cambridge</t>
         </is>
       </c>
       <c r="B49" s="9" t="n">
-        <v>74</v>
-      </c>
-      <c r="C49" s="18" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="D49" s="19" t="inlineStr">
-        <is>
-          <t>Luxury</t>
+        <v>79</v>
+      </c>
+      <c r="C49" s="16" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
         </is>
       </c>
       <c r="E49" s="10" t="n">
-        <v>1377983</v>
+        <v>995293</v>
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
@@ -1934,50 +1934,310 @@
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Lexington</t>
+          <t>Boxford</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>77</v>
-      </c>
-      <c r="C50" s="18" t="n">
-        <v>32.1</v>
-      </c>
-      <c r="D50" s="19" t="inlineStr">
-        <is>
-          <t>Luxury</t>
+        <v>74</v>
+      </c>
+      <c r="C50" s="16" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
         </is>
       </c>
       <c r="E50" s="6" t="n">
-        <v>1469802</v>
+        <v>989433</v>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="8" t="inlineStr">
         <is>
+          <t>Topsfield</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="C51" s="16" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="n">
+        <v>898745</v>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Wenham</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C52" s="16" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="n">
+        <v>938834</v>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>Lynnfield</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="C53" s="16" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="n">
+        <v>1018229</v>
+      </c>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Arlington</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="C54" s="16" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="n">
+        <v>1005584</v>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>Concord</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="C55" s="16" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>83</v>
+      </c>
+      <c r="C56" s="16" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>Nahant</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="C57" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="n">
+        <v>903532</v>
+      </c>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Manchester-by-the-Sea</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C58" s="16" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="D58" s="17" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>1183983</v>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>Belmont</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="C59" s="18" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="n">
+        <v>1377983</v>
+      </c>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Lexington</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="C60" s="18" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="D60" s="19" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="n">
+        <v>1469802</v>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
           <t>Winchester</t>
         </is>
       </c>
-      <c r="B51" s="9" t="n">
+      <c r="B61" s="9" t="n">
         <v>76</v>
       </c>
-      <c r="C51" s="18" t="n">
+      <c r="C61" s="18" t="n">
         <v>32.1</v>
       </c>
-      <c r="D51" s="19" t="inlineStr">
+      <c r="D61" s="19" t="inlineStr">
         <is>
           <t>Luxury</t>
         </is>
       </c>
-      <c r="E51" s="10" t="n">
+      <c r="E61" s="10" t="n">
         <v>1449988</v>
       </c>
-      <c r="F51" s="11" t="inlineStr">
+      <c r="F61" s="11" t="inlineStr">
         <is>
           <t>Middlesex</t>
         </is>

</xml_diff>

<commit_message>
Add civica_value_scores.xlsx to update pipeline
update_all.py now rewrites civica_value_scores.xlsx after every run —
all 80 towns, sorted by value score, with county column. Moves ZHVI
and COUNTY_MAP dicts to module scope so they're available for the
Excel write-back.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/civica_value_scores.xlsx
+++ b/civica_value_scores.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -686,14 +686,14 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Lawrence</t>
+          <t>Brockton</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>92.8</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
@@ -701,25 +701,25 @@
         </is>
       </c>
       <c r="E2" s="6" t="n">
-        <v>455876</v>
+        <v>435000</v>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Plymouth</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>Revere</t>
+          <t>Lawrence</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>90.59999999999999</v>
+        <v>92.8</v>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
@@ -727,25 +727,25 @@
         </is>
       </c>
       <c r="E3" s="10" t="n">
-        <v>440000</v>
+        <v>455876</v>
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
-          <t>Suffolk</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Haverhill</t>
+          <t>Revere</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>87.5</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
@@ -753,25 +753,25 @@
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>497568</v>
+        <v>440000</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Suffolk</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Malden</t>
+          <t>Haverhill</t>
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>83.2</v>
+        <v>87.5</v>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
@@ -779,129 +779,129 @@
         </is>
       </c>
       <c r="E5" s="10" t="n">
-        <v>545000</v>
+        <v>497568</v>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Methuen</t>
+          <t>Malden</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
         <v>74</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>80.8</v>
+        <v>83.2</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Good Value</t>
+          <t>Great Value</t>
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>561211</v>
+        <v>545000</v>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Winthrop</t>
+          <t>Quincy</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>80.2</v>
+        <v>82.5</v>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Good Value</t>
+          <t>Great Value</t>
         </is>
       </c>
       <c r="E7" s="10" t="n">
-        <v>520000</v>
+        <v>535000</v>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>Suffolk</t>
+          <t>Norfolk</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Lynn</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
         <v>70</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>79.8</v>
+        <v>82.5</v>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Good Value</t>
+          <t>Great Value</t>
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>537825</v>
+        <v>520000</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Plymouth</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Uxbridge</t>
+          <t>Weymouth</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>79.3</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Good Value</t>
+          <t>Great Value</t>
         </is>
       </c>
       <c r="E9" s="10" t="n">
-        <v>487277</v>
+        <v>530000</v>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Worcester</t>
+          <t>Norfolk</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Norwood</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>78.90000000000001</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>505101</v>
+        <v>580000</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Suffolk</t>
+          <t>Norfolk</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Everett</t>
+          <t>Methuen</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>77.5</v>
+        <v>80.8</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
@@ -935,25 +935,25 @@
         </is>
       </c>
       <c r="E11" s="10" t="n">
-        <v>530000</v>
+        <v>561211</v>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Salem</t>
+          <t>Winthrop</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C12" s="12" t="n">
-        <v>73.90000000000001</v>
+        <v>80.2</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
@@ -961,25 +961,25 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>572734</v>
+        <v>520000</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Suffolk</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Framingham</t>
+          <t>Lynn</t>
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>73.59999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
@@ -987,25 +987,25 @@
         </is>
       </c>
       <c r="E13" s="10" t="n">
-        <v>575000</v>
+        <v>537825</v>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Amesbury</t>
+          <t>Uxbridge</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>73.09999999999999</v>
+        <v>79.3</v>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
@@ -1013,25 +1013,25 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>570013</v>
+        <v>487277</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Worcester</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Merrimac</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>70.8</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
@@ -1039,25 +1039,25 @@
         </is>
       </c>
       <c r="E15" s="10" t="n">
-        <v>597359</v>
+        <v>505101</v>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Suffolk</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Stoneham</t>
+          <t>Plymouth</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>70.2</v>
+        <v>78.3</v>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
@@ -1065,25 +1065,25 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>690000</v>
+        <v>540000</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Plymouth</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Danvers</t>
+          <t>Everett</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>69.09999999999999</v>
+        <v>77.5</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
@@ -1091,25 +1091,25 @@
         </is>
       </c>
       <c r="E17" s="10" t="n">
-        <v>674241</v>
+        <v>530000</v>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Woburn</t>
+          <t>Braintree</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C18" s="12" t="n">
-        <v>67.90000000000001</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
@@ -1117,25 +1117,25 @@
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>704405</v>
+        <v>640000</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Norfolk</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Saugus</t>
+          <t>Salem</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>67.8</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="E19" s="10" t="n">
-        <v>650624</v>
+        <v>572734</v>
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
@@ -1154,14 +1154,14 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Salisbury</t>
+          <t>Framingham</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C20" s="12" t="n">
-        <v>67.59999999999999</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>589785</v>
+        <v>575000</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Groveland</t>
+          <t>Amesbury</t>
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C21" s="12" t="n">
-        <v>66.2</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="E21" s="10" t="n">
-        <v>648353</v>
+        <v>570013</v>
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
@@ -1206,14 +1206,14 @@
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Merrimac</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C22" s="12" t="n">
-        <v>65.59999999999999</v>
+        <v>70.8</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1221,59 +1221,59 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>720000</v>
+        <v>597359</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Suffolk</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Beverly</t>
+          <t>Hanover</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C23" s="14" t="n">
-        <v>64.3</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>Fair Market</t>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E23" s="10" t="n">
-        <v>696077</v>
+        <v>660000</v>
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Plymouth</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Natick</t>
+          <t>Stoneham</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C24" s="14" t="n">
-        <v>63.3</v>
+        <v>70.2</v>
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>Fair Market</t>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>775000</v>
+        <v>690000</v>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
@@ -1284,74 +1284,74 @@
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Burlington</t>
+          <t>Canton</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C25" s="14" t="n">
-        <v>63.2</v>
+        <v>69.8</v>
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>Fair Market</t>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E25" s="10" t="n">
-        <v>824833</v>
+        <v>720000</v>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Norfolk</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Wakefield</t>
+          <t>Danvers</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C26" s="14" t="n">
-        <v>63.2</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>Fair Market</t>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>756484</v>
+        <v>674241</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Waltham</t>
+          <t>Woburn</t>
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C27" s="14" t="n">
-        <v>63</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>Fair Market</t>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E27" s="10" t="n">
-        <v>720000</v>
+        <v>704405</v>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
@@ -1362,22 +1362,22 @@
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>North Andover</t>
+          <t>Saugus</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C28" s="14" t="n">
-        <v>60.4</v>
+        <v>67.8</v>
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>Fair Market</t>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>760639</v>
+        <v>650624</v>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
@@ -1388,48 +1388,48 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Medford</t>
+          <t>Salisbury</t>
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="C29" s="14" t="n">
-        <v>58.6</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>Fair Market</t>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E29" s="10" t="n">
-        <v>784462</v>
+        <v>589785</v>
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Peabody</t>
+          <t>Groveland</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="C30" s="14" t="n">
-        <v>58.3</v>
+        <v>66.2</v>
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>Fair Market</t>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>652390</v>
+        <v>648353</v>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
@@ -1440,66 +1440,66 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Georgetown</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="C31" s="14" t="n">
-        <v>57.9</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>Fair Market</t>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E31" s="10" t="n">
-        <v>708796</v>
+        <v>720000</v>
       </c>
       <c r="F31" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Suffolk</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Watertown</t>
+          <t>Marshfield</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="C32" s="14" t="n">
-        <v>57.7</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>Fair Market</t>
+          <t>Good Value</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>840000</v>
+        <v>640000</v>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Plymouth</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Acton</t>
+          <t>Dedham</t>
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C33" s="14" t="n">
-        <v>57.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
@@ -1507,25 +1507,25 @@
         </is>
       </c>
       <c r="E33" s="10" t="n">
-        <v>840000</v>
+        <v>690000</v>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Norfolk</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Ipswich</t>
+          <t>Beverly</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C34" s="14" t="n">
-        <v>57.4</v>
+        <v>64.3</v>
       </c>
       <c r="D34" s="15" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>790546</v>
+        <v>696077</v>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
@@ -1544,14 +1544,14 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>Natick</t>
         </is>
       </c>
       <c r="B35" s="9" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C35" s="14" t="n">
-        <v>57.4</v>
+        <v>63.3</v>
       </c>
       <c r="D35" s="15" t="inlineStr">
         <is>
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="E35" s="10" t="n">
-        <v>844034</v>
+        <v>775000</v>
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
@@ -1570,14 +1570,14 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Rowley</t>
+          <t>Burlington</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="C36" s="14" t="n">
-        <v>56.8</v>
+        <v>63.2</v>
       </c>
       <c r="D36" s="15" t="inlineStr">
         <is>
@@ -1585,25 +1585,25 @@
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>733628</v>
+        <v>824833</v>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>Gloucester</t>
+          <t>Wakefield</t>
         </is>
       </c>
       <c r="B37" s="9" t="n">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="C37" s="14" t="n">
-        <v>56.6</v>
+        <v>63.2</v>
       </c>
       <c r="D37" s="15" t="inlineStr">
         <is>
@@ -1611,25 +1611,25 @@
         </is>
       </c>
       <c r="E37" s="10" t="n">
-        <v>693415</v>
+        <v>756484</v>
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Andover</t>
+          <t>Waltham</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="C38" s="14" t="n">
-        <v>55.8</v>
+        <v>63</v>
       </c>
       <c r="D38" s="15" t="inlineStr">
         <is>
@@ -1637,25 +1637,25 @@
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>911128</v>
+        <v>720000</v>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>Swampscott</t>
+          <t>North Andover</t>
         </is>
       </c>
       <c r="B39" s="9" t="n">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C39" s="14" t="n">
-        <v>55.4</v>
+        <v>60.4</v>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
@@ -1663,7 +1663,7 @@
         </is>
       </c>
       <c r="E39" s="10" t="n">
-        <v>763080</v>
+        <v>760639</v>
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
@@ -1674,14 +1674,14 @@
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Middleton</t>
+          <t>Medford</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C40" s="14" t="n">
-        <v>55.4</v>
+        <v>58.6</v>
       </c>
       <c r="D40" s="15" t="inlineStr">
         <is>
@@ -1689,25 +1689,25 @@
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>819582</v>
+        <v>784462</v>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>Hamilton</t>
+          <t>Peabody</t>
         </is>
       </c>
       <c r="B41" s="9" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="C41" s="14" t="n">
-        <v>53.3</v>
+        <v>58.3</v>
       </c>
       <c r="D41" s="15" t="inlineStr">
         <is>
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="E41" s="10" t="n">
-        <v>827397</v>
+        <v>652390</v>
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
@@ -1726,14 +1726,14 @@
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Newbury</t>
+          <t>Georgetown</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C42" s="14" t="n">
-        <v>52.3</v>
+        <v>57.9</v>
       </c>
       <c r="D42" s="15" t="inlineStr">
         <is>
@@ -1741,7 +1741,7 @@
         </is>
       </c>
       <c r="E42" s="6" t="n">
-        <v>844611</v>
+        <v>708796</v>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
@@ -1752,14 +1752,14 @@
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>Rockport</t>
+          <t>Watertown</t>
         </is>
       </c>
       <c r="B43" s="9" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C43" s="14" t="n">
-        <v>52.2</v>
+        <v>57.7</v>
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
@@ -1767,25 +1767,25 @@
         </is>
       </c>
       <c r="E43" s="10" t="n">
-        <v>834071</v>
+        <v>840000</v>
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Newburyport</t>
+          <t>Acton</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C44" s="14" t="n">
-        <v>51.5</v>
+        <v>57.7</v>
       </c>
       <c r="D44" s="15" t="inlineStr">
         <is>
@@ -1793,25 +1793,25 @@
         </is>
       </c>
       <c r="E44" s="6" t="n">
-        <v>845604</v>
+        <v>840000</v>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Somerville</t>
+          <t>Ipswich</t>
         </is>
       </c>
       <c r="B45" s="9" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C45" s="14" t="n">
-        <v>51.5</v>
+        <v>57.4</v>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
@@ -1819,25 +1819,25 @@
         </is>
       </c>
       <c r="E45" s="10" t="n">
-        <v>892143</v>
+        <v>790546</v>
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Marblehead</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B46" s="3" t="n">
         <v>79</v>
       </c>
       <c r="C46" s="14" t="n">
-        <v>50.5</v>
+        <v>57.4</v>
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
@@ -1845,25 +1845,25 @@
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>959425</v>
+        <v>844034</v>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>West Newbury</t>
+          <t>Norwell</t>
         </is>
       </c>
       <c r="B47" s="9" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C47" s="14" t="n">
-        <v>50.5</v>
+        <v>57</v>
       </c>
       <c r="D47" s="15" t="inlineStr">
         <is>
@@ -1871,25 +1871,25 @@
         </is>
       </c>
       <c r="E47" s="10" t="n">
-        <v>861236</v>
+        <v>850000</v>
       </c>
       <c r="F47" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Plymouth</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Rowley</t>
         </is>
       </c>
       <c r="B48" s="3" t="n">
         <v>68</v>
       </c>
       <c r="C48" s="14" t="n">
-        <v>50.4</v>
+        <v>56.8</v>
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="E48" s="6" t="n">
-        <v>827029</v>
+        <v>733628</v>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
@@ -1908,48 +1908,48 @@
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>Cambridge</t>
+          <t>Gloucester</t>
         </is>
       </c>
       <c r="B49" s="9" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="C49" s="16" t="n">
-        <v>48.7</v>
+        <v>56.6</v>
       </c>
       <c r="D49" s="17" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E49" s="10" t="n">
-        <v>995293</v>
+        <v>693415</v>
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Boxford</t>
+          <t>Andover</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="C50" s="16" t="n">
-        <v>45.9</v>
+        <v>55.8</v>
       </c>
       <c r="D50" s="17" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E50" s="6" t="n">
-        <v>989433</v>
+        <v>911128</v>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
@@ -1960,22 +1960,22 @@
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>Topsfield</t>
+          <t>Swampscott</t>
         </is>
       </c>
       <c r="B51" s="9" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C51" s="16" t="n">
-        <v>45.7</v>
+        <v>55.4</v>
       </c>
       <c r="D51" s="17" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E51" s="10" t="n">
-        <v>898745</v>
+        <v>763080</v>
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
@@ -1986,22 +1986,22 @@
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Wenham</t>
+          <t>Middleton</t>
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C52" s="16" t="n">
-        <v>45.7</v>
+        <v>55.4</v>
       </c>
       <c r="D52" s="17" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>938834</v>
+        <v>819582</v>
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
@@ -2012,22 +2012,22 @@
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>Lynnfield</t>
+          <t>Hamilton</t>
         </is>
       </c>
       <c r="B53" s="9" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C53" s="16" t="n">
-        <v>45.2</v>
+        <v>53.3</v>
       </c>
       <c r="D53" s="17" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E53" s="10" t="n">
-        <v>1018229</v>
+        <v>827397</v>
       </c>
       <c r="F53" s="11" t="inlineStr">
         <is>
@@ -2038,208 +2038,728 @@
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Arlington</t>
+          <t>Newbury</t>
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C54" s="16" t="n">
-        <v>45.1</v>
+        <v>52.3</v>
       </c>
       <c r="D54" s="17" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E54" s="6" t="n">
-        <v>1005584</v>
+        <v>844611</v>
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>Concord</t>
+          <t>Rockport</t>
         </is>
       </c>
       <c r="B55" s="9" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="C55" s="16" t="n">
-        <v>44.6</v>
+        <v>52.2</v>
       </c>
       <c r="D55" s="17" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E55" s="10" t="n">
-        <v>1100000</v>
+        <v>834071</v>
       </c>
       <c r="F55" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Newton</t>
+          <t>Newburyport</t>
         </is>
       </c>
       <c r="B56" s="3" t="n">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="C56" s="16" t="n">
-        <v>42.4</v>
+        <v>51.5</v>
       </c>
       <c r="D56" s="17" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E56" s="6" t="n">
-        <v>1200000</v>
+        <v>845604</v>
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>Nahant</t>
+          <t>Somerville</t>
         </is>
       </c>
       <c r="B57" s="9" t="n">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="C57" s="16" t="n">
-        <v>40</v>
+        <v>51.5</v>
       </c>
       <c r="D57" s="17" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E57" s="10" t="n">
-        <v>903532</v>
+        <v>892143</v>
       </c>
       <c r="F57" s="11" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Middlesex</t>
         </is>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Manchester-by-the-Sea</t>
+          <t>Scituate</t>
         </is>
       </c>
       <c r="B58" s="3" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C58" s="16" t="n">
-        <v>36.2</v>
+        <v>51.2</v>
       </c>
       <c r="D58" s="17" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E58" s="6" t="n">
-        <v>1183983</v>
+        <v>850000</v>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>Essex</t>
+          <t>Plymouth</t>
         </is>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>Belmont</t>
+          <t>Marblehead</t>
         </is>
       </c>
       <c r="B59" s="9" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C59" s="18" t="n">
-        <v>32.9</v>
+        <v>50.5</v>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Luxury</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E59" s="10" t="n">
-        <v>1377983</v>
+        <v>959425</v>
       </c>
       <c r="F59" s="11" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Lexington</t>
+          <t>West Newbury</t>
         </is>
       </c>
       <c r="B60" s="3" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C60" s="18" t="n">
-        <v>32.1</v>
+        <v>50.5</v>
       </c>
       <c r="D60" s="19" t="inlineStr">
         <is>
-          <t>Luxury</t>
+          <t>Fair Market</t>
         </is>
       </c>
       <c r="E60" s="6" t="n">
-        <v>1469802</v>
+        <v>861236</v>
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>Middlesex</t>
+          <t>Essex</t>
         </is>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="8" t="inlineStr">
         <is>
+          <t>Essex</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="C61" s="18" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>Fair Market</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="n">
+        <v>827029</v>
+      </c>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Milton</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>79</v>
+      </c>
+      <c r="C62" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>970000</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Norfolk</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Cambridge</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>79</v>
+      </c>
+      <c r="C63" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>995293</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Boxford</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>74</v>
+      </c>
+      <c r="C64" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>989433</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Topsfield</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>67</v>
+      </c>
+      <c r="C65" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>898745</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Wenham</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>70</v>
+      </c>
+      <c r="C66" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>938834</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Duxbury</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>73</v>
+      </c>
+      <c r="C67" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>980000</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Plymouth</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Lynnfield</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>75</v>
+      </c>
+      <c r="C68" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1018229</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Arlington</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>74</v>
+      </c>
+      <c r="C69" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>1005584</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Concord</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>80</v>
+      </c>
+      <c r="C70" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Hingham</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>77</v>
+      </c>
+      <c r="C71" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Plymouth</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>83</v>
+      </c>
+      <c r="C72" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Nahant</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>59</v>
+      </c>
+      <c r="C73" t="n">
+        <v>40</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>903532</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Needham</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>81</v>
+      </c>
+      <c r="C74" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>1250000</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Norfolk</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Manchester-by-the-Sea</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>70</v>
+      </c>
+      <c r="C75" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>1183983</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Cohasset</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>68</v>
+      </c>
+      <c r="C76" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>1250000</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Plymouth</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Brookline</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>78</v>
+      </c>
+      <c r="C77" t="n">
+        <v>33</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Norfolk</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Belmont</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>74</v>
+      </c>
+      <c r="C78" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1377983</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Lexington</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>77</v>
+      </c>
+      <c r="C79" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>1469802</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>Winchester</t>
         </is>
       </c>
-      <c r="B61" s="9" t="n">
+      <c r="B80" t="n">
         <v>76</v>
       </c>
-      <c r="C61" s="18" t="n">
+      <c r="C80" t="n">
         <v>32.1</v>
       </c>
-      <c r="D61" s="19" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>Luxury</t>
         </is>
       </c>
-      <c r="E61" s="10" t="n">
+      <c r="E80" t="n">
         <v>1449988</v>
       </c>
-      <c r="F61" s="11" t="inlineStr">
+      <c r="F80" t="inlineStr">
         <is>
           <t>Middlesex</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Wellesley</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>80</v>
+      </c>
+      <c r="C81" t="n">
+        <v>28</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Luxury</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>1750000</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Norfolk</t>
         </is>
       </c>
     </row>

</xml_diff>